<commit_message>
ui pop up changes
</commit_message>
<xml_diff>
--- a/invalid_leads.xlsx
+++ b/invalid_leads.xlsx
@@ -20,14 +20,9 @@
     <author>Validation</author>
   </authors>
   <commentList>
-    <comment ref="D3" authorId="1">
+    <comment ref="B3" authorId="1">
       <text>
-        <t>Invalid Mobile Number</t>
-      </text>
-    </comment>
-    <comment ref="F3" authorId="1">
-      <text>
-        <t>Invalid GSTIN</t>
+        <t>Invalid First Name</t>
       </text>
     </comment>
     <comment ref="B4" authorId="1">
@@ -35,12 +30,27 @@
         <t>Invalid First Name</t>
       </text>
     </comment>
-    <comment ref="C4" authorId="1">
+    <comment ref="B5" authorId="1">
+      <text>
+        <t>Invalid First Name</t>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="1">
+      <text>
+        <t>Invalid GSTIN</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="1">
+      <text>
+        <t>Invalid First Name</t>
+      </text>
+    </comment>
+    <comment ref="C6" authorId="1">
       <text>
         <t>Invalid Last Name</t>
       </text>
     </comment>
-    <comment ref="D4" authorId="1">
+    <comment ref="D6" authorId="1">
       <text>
         <t>Invalid Mobile Number</t>
       </text>
@@ -50,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
   <si>
     <t>Products</t>
   </si>
@@ -103,25 +113,40 @@
     <t>Description (O)</t>
   </si>
   <si>
-    <t>rohan</t>
+    <t>user1</t>
   </si>
   <si>
-    <t>Rhote</t>
+    <t>userlastname</t>
   </si>
   <si>
-    <t>83457952121</t>
+    <t>8308736626</t>
   </si>
   <si>
-    <t>rohan.rote@gmail.com</t>
+    <t>user1@gmail.com</t>
+  </si>
+  <si>
+    <t>SGTE2IRQ5GN67SW</t>
+  </si>
+  <si>
+    <t>silicon vally</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>user2</t>
+  </si>
+  <si>
+    <t>8357952121</t>
+  </si>
+  <si>
+    <t>user2@gmail.com</t>
   </si>
   <si>
     <t>ANDTE23</t>
   </si>
   <si>
     <t>washinton dc</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>user3</t>
@@ -752,23 +777,23 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s" s="14">
         <v>17</v>
       </c>
       <c r="C3" t="s" s="0">
         <v>18</v>
       </c>
-      <c r="D3" t="s" s="14">
+      <c r="D3" t="s" s="0">
         <v>19</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>20</v>
       </c>
-      <c r="F3" t="s" s="14">
+      <c r="F3" t="s" s="0">
         <v>21</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H3" t="s" s="0">
         <v>22</v>
@@ -779,35 +804,81 @@
     </row>
     <row r="4">
       <c r="B4" t="s" s="14">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="s" s="14">
         <v>24</v>
       </c>
-      <c r="C4" t="s" s="14">
+      <c r="C5" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="D4" t="s" s="14">
+      <c r="E5" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="E4" t="s" s="0">
+      <c r="F5" t="s" s="14">
         <v>27</v>
       </c>
-      <c r="F4" t="s" s="0">
+      <c r="G5" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="H5" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="G4" t="s" s="0">
+      <c r="I5" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="s" s="14">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s" s="14">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s" s="14">
+        <v>31</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="H4" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="I4" t="s" s="0">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="G5" s="13"/>
-    </row>
-    <row r="6">
-      <c r="G6" s="13"/>
+      <c r="H6" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>35</v>
+      </c>
     </row>
     <row r="7">
       <c r="G7" s="13"/>

</xml_diff>